<commit_message>
added selectNext, selectAll, and clearAll
</commit_message>
<xml_diff>
--- a/static_content/jobs/jobs.xlsx
+++ b/static_content/jobs/jobs.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="113">
   <si>
     <t>role</t>
   </si>
@@ -55,10 +55,10 @@
     <t>darkcyan</t>
   </si>
   <si>
-    <t>#008b8b</t>
-  </si>
-  <si>
-    <t>black</t>
+    <t>#006688</t>
+  </si>
+  <si>
+    <t>white</t>
   </si>
   <si>
     <t>• Working as a consulting data engineer in the data cyber security team of the [Cigna Group](url).</t>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>#0000ff</t>
-  </si>
-  <si>
-    <t>white</t>
   </si>
   <si>
     <t>• Worked as a consulting data engineer in the analytics team of [Warner Brothers Interactive Entertainment](url) Division.
@@ -88,7 +85,7 @@
     <t>mediumblue</t>
   </si>
   <si>
-    <t>#0000cd</t>
+    <t>#4400cd</t>
   </si>
   <si>
     <t>• Worked as a consulting data engineer for [Angel Studios](url], a streaming media service that offers family-friendly entertainment that amplifies light, with titles including The Chosen, Dry Bar Comedy, and Tuttle Twins.
@@ -132,7 +129,7 @@
     <t xml:space="preserve">Senior Data Engineer </t>
   </si>
   <si>
-    <t>SeniorLiink</t>
+    <t>b</t>
   </si>
   <si>
     <t>maroon</t>
@@ -176,6 +173,9 @@
   </si>
   <si>
     <t>#ff4500</t>
+  </si>
+  <si>
+    <t>black</t>
   </si>
   <si>
     <t>• Co-founded a company that envisioned building a web destination where users could easily record and share their favorite pieces of content like facts, authored stories, quotes, articles, chapters, or personal thoughts, as a way of concretely defining their personal mindset.
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t xml:space="preserve">BuildingBlocks LLC </t>
+  </si>
+  <si>
+    <t>#008b8b</t>
   </si>
   <si>
     <t>• As lead software developer, built a CD-ROM-based home design application for selecting premium home design products for previewing in the context of images of any household rooms. 
@@ -256,6 +259,9 @@
   </si>
   <si>
     <t>BYU</t>
+  </si>
+  <si>
+    <t>#0000cd</t>
   </si>
   <si>
     <t>• Masters of Science degree, Brigham Young University, Provo, Utah
@@ -1023,7 +1029,7 @@
         <v>45047</v>
       </c>
       <c r="D2" s="6">
-        <v>45108</v>
+        <v>45139</v>
       </c>
       <c r="E2" s="7">
         <v>3</v>
@@ -1066,10 +1072,10 @@
       </c>
       <c r="H3" s="10"/>
       <c r="I3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>20</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="157.5">
@@ -1077,7 +1083,7 @@
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="6">
         <v>44501</v>
@@ -1089,17 +1095,17 @@
         <v>1</v>
       </c>
       <c r="F4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>23</v>
       </c>
       <c r="H4" s="11"/>
       <c r="I4" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="88.5">
@@ -1107,7 +1113,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="6">
         <v>44136</v>
@@ -1119,25 +1125,25 @@
         <v>2</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="60.75">
       <c r="A6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="C6" s="6">
         <v>43770</v>
@@ -1149,25 +1155,25 @@
         <v>1</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="H6" s="13"/>
       <c r="I6" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J6" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="212.25">
+      <c r="A7" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="168">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>35</v>
       </c>
       <c r="C7" s="6">
         <v>42795</v>
@@ -1179,25 +1185,25 @@
         <v>2</v>
       </c>
       <c r="F7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="H7" s="14"/>
       <c r="I7" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J7" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="88.5">
+      <c r="A8" s="5" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="75.75">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="C8" s="6">
         <v>42705</v>
@@ -1209,25 +1215,25 @@
         <v>1</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>42</v>
       </c>
       <c r="H8" s="15"/>
       <c r="I8" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J8" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="212.25">
+      <c r="A9" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="168">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="C9" s="6">
         <v>40575</v>
@@ -1239,22 +1245,22 @@
         <v>2</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>47</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="156.75">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="184.5">
       <c r="A10" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>49</v>
@@ -1276,7 +1282,7 @@
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>52</v>
@@ -1284,7 +1290,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="133.5">
       <c r="A11" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>53</v>
@@ -1306,7 +1312,7 @@
       </c>
       <c r="H11" s="18"/>
       <c r="I11" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>56</v>
@@ -1332,22 +1338,22 @@
         <v>12</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="H12" s="8"/>
       <c r="I12" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="214.5">
       <c r="A13" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C13" s="6">
         <v>33117</v>
@@ -1366,18 +1372,18 @@
       </c>
       <c r="H13" s="10"/>
       <c r="I13" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="179.25">
       <c r="A14" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="6">
         <v>32021</v>
@@ -1389,25 +1395,25 @@
         <v>2</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="40.5">
       <c r="A15" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C15" s="6">
         <v>32295</v>
@@ -1419,25 +1425,25 @@
         <v>3</v>
       </c>
       <c r="F15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="H15" s="12"/>
       <c r="I15" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
       <c r="A16" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" s="6">
         <v>30926</v>
@@ -1449,25 +1455,25 @@
         <v>2</v>
       </c>
       <c r="F16" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="H16" s="13"/>
       <c r="I16" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="40.5">
       <c r="A17" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C17" s="6">
         <v>30682</v>
@@ -1479,25 +1485,25 @@
         <v>1</v>
       </c>
       <c r="F17" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="29.25">
       <c r="A18" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C18" s="6">
         <v>30133</v>
@@ -1509,25 +1515,25 @@
         <v>3</v>
       </c>
       <c r="F18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>42</v>
       </c>
       <c r="H18" s="15"/>
       <c r="I18" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
       <c r="A19" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C19" s="6">
         <v>29830</v>
@@ -1539,25 +1545,25 @@
         <v>2</v>
       </c>
       <c r="F19" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>47</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="40.5">
       <c r="A20" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C20" s="6">
         <v>29677</v>
@@ -1576,18 +1582,18 @@
       </c>
       <c r="H20" s="17"/>
       <c r="I20" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="41.25">
       <c r="A21" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C21" s="6">
         <v>28369</v>
@@ -1599,25 +1605,25 @@
         <v>1</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="109.5">
       <c r="A22" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C22" s="6">
         <v>39417</v>
@@ -1629,25 +1635,25 @@
         <v>2</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H22" s="20"/>
       <c r="I22" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J22" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="75.75">
       <c r="A23" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C23" s="6">
         <v>38749</v>
@@ -1659,25 +1665,25 @@
         <v>2</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H23" s="22"/>
       <c r="I23" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="63.75">
       <c r="A24" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C24" s="6">
         <v>38384</v>
@@ -1689,25 +1695,25 @@
         <v>2</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H24" s="23"/>
       <c r="I24" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="63.75">
       <c r="A25" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C25" s="6">
         <v>38018</v>
@@ -1719,25 +1725,25 @@
         <v>2</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H25" s="24"/>
       <c r="I25" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="87.75">
       <c r="A26" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C26" s="6">
         <v>37681</v>
@@ -1749,17 +1755,17 @@
         <v>2</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H26" s="25"/>
       <c r="I26" s="5" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bizcards are now animating to the top, but not staying there - animationendlistener not firing
</commit_message>
<xml_diff>
--- a/static_content/jobs/jobs.xlsx
+++ b/static_content/jobs/jobs.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10709"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sbecker11/workspace-modules/flock-of-postcards/static_content/jobs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FC39CB-B793-1647-83E7-3F9384DC1CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-52600" yWindow="4580" windowWidth="18200" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="jobs"/>
+    <sheet name="jobs" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -56,9 +62,6 @@
   </si>
   <si>
     <t>#006688</t>
-  </si>
-  <si>
-    <t>white</t>
   </si>
   <si>
     <t>• Working as a consulting data engineer in the data cyber security team of the [Cigna Group](url).</t>
@@ -173,9 +176,6 @@
   </si>
   <si>
     <t>#ff4500</t>
-  </si>
-  <si>
-    <t>black</t>
   </si>
   <si>
     <t>• Co-founded a company that envisioned building a web destination where users could easily record and share their favorite pieces of content like facts, authored stories, quotes, articles, chapters, or personal thoughts, as a way of concretely defining their personal mindset.
@@ -428,13 +428,19 @@
 •  Used [Java](url), [ObjectDesign](url), [JavaScript ES3](url), [MySQL 4](url), and [Adobe Photoshop v5.0](url). 
 </t>
   </si>
+  <si>
+    <t>#FFFFFF</t>
+  </si>
+  <si>
+    <t>#000000</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -467,22 +473,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF008b8b"/>
+        <fgColor rgb="FF008B8B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0000ff"/>
+        <fgColor rgb="FF0000FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF0000cd"/>
+        <fgColor rgb="FF0000CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF8a2be2"/>
+        <fgColor rgb="FF8A2BE2"/>
       </patternFill>
     </fill>
     <fill>
@@ -497,17 +503,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFdc143c"/>
+        <fgColor rgb="FFDC143C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFff4500"/>
+        <fgColor rgb="FFFF4500"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffa500"/>
+        <fgColor rgb="FFFFA500"/>
       </patternFill>
     </fill>
     <fill>
@@ -517,32 +523,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffd700"/>
+        <fgColor rgb="FFFFD700"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffff00"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00ff00"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF32cd32"/>
+        <fgColor rgb="FF32CD32"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF6b8e23"/>
+        <fgColor rgb="FF6B8E23"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF228b22"/>
+        <fgColor rgb="FF228B22"/>
       </patternFill>
     </fill>
   </fills>
@@ -581,103 +587,106 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="30">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="15" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="16" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="17" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -688,10 +697,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -729,71 +738,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -821,7 +830,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -844,11 +853,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -857,13 +866,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -873,7 +882,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -882,7 +891,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -891,7 +900,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -899,10 +908,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -967,26 +976,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" style="26" width="22.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="26" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="27" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="27" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="28" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="26" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="26" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="26" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="26" width="10.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="29" width="96.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="22.1640625" style="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.6640625" style="26" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.83203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" style="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="10.83203125" style="26" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="96" style="29" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1018,7 +1023,7 @@
         <v>9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>10</v>
       </c>
@@ -1042,18 +1047,18 @@
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="J2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="129.75">
+    </row>
+    <row r="3" spans="1:10" ht="129.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" s="6">
         <v>44805</v>
@@ -1065,25 +1070,25 @@
         <v>2</v>
       </c>
       <c r="F3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>18</v>
       </c>
       <c r="H3" s="10"/>
       <c r="I3" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="157.5">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="157.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4" s="6">
         <v>44501</v>
@@ -1095,25 +1100,25 @@
         <v>1</v>
       </c>
       <c r="F4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>22</v>
       </c>
       <c r="H4" s="11"/>
       <c r="I4" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="88.5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="6">
         <v>44136</v>
@@ -1125,25 +1130,25 @@
         <v>2</v>
       </c>
       <c r="F5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="H5" s="12"/>
       <c r="I5" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J5" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="60.75">
-      <c r="A6" s="5" t="s">
+      <c r="B6" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="C6" s="6">
         <v>43770</v>
@@ -1155,25 +1160,25 @@
         <v>1</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>31</v>
       </c>
       <c r="H6" s="13"/>
       <c r="I6" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J6" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="212.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="212.25">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>34</v>
       </c>
       <c r="C7" s="6">
         <v>42795</v>
@@ -1185,25 +1190,25 @@
         <v>2</v>
       </c>
       <c r="F7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="H7" s="14"/>
       <c r="I7" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J7" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="88.5">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="C8" s="6">
         <v>42705</v>
@@ -1215,25 +1220,25 @@
         <v>1</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="H8" s="15"/>
       <c r="I8" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J8" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="212.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="212.25">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="C9" s="6">
         <v>40575</v>
@@ -1245,25 +1250,25 @@
         <v>2</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="H9" s="16"/>
       <c r="I9" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="184.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="184.5">
-      <c r="A10" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>49</v>
       </c>
       <c r="C10" s="6">
         <v>37561</v>
@@ -1275,25 +1280,25 @@
         <v>1</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="133.5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="133.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C11" s="6">
         <v>35827</v>
@@ -1305,25 +1310,25 @@
         <v>1</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H11" s="18"/>
       <c r="I11" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J11" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>56</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="75.75">
-      <c r="A12" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="C12" s="6">
         <v>35217</v>
@@ -1338,22 +1343,22 @@
         <v>12</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H12" s="8"/>
       <c r="I12" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J12" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="214.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="214.5">
-      <c r="A13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="C13" s="6">
         <v>33117</v>
@@ -1365,25 +1370,25 @@
         <v>2</v>
       </c>
       <c r="F13" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>18</v>
       </c>
       <c r="H13" s="10"/>
       <c r="I13" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J13" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="179.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="179.25">
-      <c r="A14" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="C14" s="6">
         <v>32021</v>
@@ -1395,25 +1400,25 @@
         <v>2</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J14" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="40.5">
-      <c r="A15" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="C15" s="6">
         <v>32295</v>
@@ -1425,25 +1430,25 @@
         <v>3</v>
       </c>
       <c r="F15" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>26</v>
       </c>
       <c r="H15" s="12"/>
       <c r="I15" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="17.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C16" s="6">
         <v>30926</v>
@@ -1455,25 +1460,25 @@
         <v>2</v>
       </c>
       <c r="F16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>31</v>
       </c>
       <c r="H16" s="13"/>
       <c r="I16" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J16" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="40.5">
-      <c r="A17" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>74</v>
       </c>
       <c r="C17" s="6">
         <v>30682</v>
@@ -1485,25 +1490,25 @@
         <v>1</v>
       </c>
       <c r="F17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="H17" s="14"/>
       <c r="I17" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J17" s="9" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="29.25">
-      <c r="A18" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="C18" s="6">
         <v>30133</v>
@@ -1515,25 +1520,25 @@
         <v>3</v>
       </c>
       <c r="F18" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="H18" s="15"/>
       <c r="I18" s="5" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="17.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C19" s="6">
         <v>29830</v>
@@ -1545,25 +1550,25 @@
         <v>2</v>
       </c>
       <c r="F19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="H19" s="16"/>
       <c r="I19" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J19" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="40.5">
-      <c r="A20" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>82</v>
       </c>
       <c r="C20" s="6">
         <v>29677</v>
@@ -1575,25 +1580,25 @@
         <v>1</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H20" s="17"/>
       <c r="I20" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J20" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="41.25">
-      <c r="A21" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="C21" s="6">
         <v>28369</v>
@@ -1605,25 +1610,25 @@
         <v>1</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J21" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="109.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="109.5">
-      <c r="A22" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>90</v>
       </c>
       <c r="C22" s="6">
         <v>39417</v>
@@ -1635,25 +1640,25 @@
         <v>2</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H22" s="20"/>
       <c r="I22" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J22" s="21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="75.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="75.75">
-      <c r="A23" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>95</v>
       </c>
       <c r="C23" s="6">
         <v>38749</v>
@@ -1665,25 +1670,25 @@
         <v>2</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H23" s="22"/>
       <c r="I23" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J23" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" s="5" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="63.75">
-      <c r="A24" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>100</v>
       </c>
       <c r="C24" s="6">
         <v>38384</v>
@@ -1695,25 +1700,25 @@
         <v>2</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H24" s="23"/>
       <c r="I24" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J24" s="9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="63.75">
-      <c r="A25" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="C25" s="6">
         <v>38018</v>
@@ -1725,25 +1730,25 @@
         <v>2</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H25" s="24"/>
       <c r="I25" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="87.75">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="87.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C26" s="6">
         <v>37681</v>
@@ -1755,17 +1760,17 @@
         <v>2</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H26" s="25"/>
       <c r="I26" s="5" t="s">
-        <v>47</v>
+        <v>112</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
auto-computing timeline min-max years, and interpolating CURRENT_DATE  in xlsx file
</commit_message>
<xml_diff>
--- a/static_content/jobs/jobs.xlsx
+++ b/static_content/jobs/jobs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10709"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11110"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sbecker11/workspace-modules/flock-of-postcards/static_content/jobs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sbecker11/workspace-parallax/flock-of-postcards/static_content/jobs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FC39CB-B793-1647-83E7-3F9384DC1CC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B494B0-C665-7B45-A8C0-7C960F5B24BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-52600" yWindow="4580" windowWidth="18200" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="114">
   <si>
     <t>role</t>
   </si>
@@ -433,6 +433,9 @@
   </si>
   <si>
     <t>#000000</t>
+  </si>
+  <si>
+    <t>CURRENT_DATE</t>
   </si>
 </sst>
 </file>
@@ -985,7 +988,8 @@
   <cols>
     <col min="1" max="1" width="22.1640625" style="26" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" style="26" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.83203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13" style="27" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" style="28" bestFit="1" customWidth="1"/>
     <col min="6" max="9" width="10.83203125" style="26" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="96" style="29" bestFit="1" customWidth="1"/>
@@ -1033,8 +1037,8 @@
       <c r="C2" s="6">
         <v>45047</v>
       </c>
-      <c r="D2" s="6">
-        <v>45139</v>
+      <c r="D2" s="6" t="s">
+        <v>113</v>
       </c>
       <c r="E2" s="7">
         <v>3</v>

</xml_diff>

<commit_message>
index.html confirmIconTags, fixed bizcard jobStart/EndStrs, logAllBizcardDivs uniques sorted, keeps, ignores, sankey diagram, dateSortedBizcards, welcomeAlert widened and centered, jobs.xlsx trimmed and normalized
</commit_message>
<xml_diff>
--- a/static_content/jobs/jobs.xlsx
+++ b/static_content/jobs/jobs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sbecker11/workspace-parallax/flock-of-postcards/static_content/jobs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08119FD-2A06-034A-9003-435380700CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF515D2-9D53-444D-B085-7027FFF1656B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="2560" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-65380" yWindow="4260" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
@@ -61,9 +61,6 @@
     <t>#006688</t>
   </si>
   <si>
-    <t>Warner Brothers Interactive Entertainment</t>
-  </si>
-  <si>
     <t>blue</t>
   </si>
   <si>
@@ -77,9 +74,6 @@
   </si>
   <si>
     <t>#4400cd</t>
-  </si>
-  <si>
-    <t>Greenseed Tech</t>
   </si>
   <si>
     <t>blueviolet</t>
@@ -268,10 +262,59 @@
   <si>
     <t>• [Intrusic LLC](https://www.crunchbase.com/organization/intrusic) built real-time network monitoring systems that identified external and internal network intrusion attempts
 • As a Sierra Vista Group architech, I helped design and develop an approach for buffering live streaming network traffic for asynchronous package processing. 
-• Used [Debian Linux](https://www.debian.org/), [C programming language](https://www.cprogramming.com/books/ritchie.html), and [Visio](https://www.microsoft.com/en-us/microsoft-365/visio/flowchart-software).</t>
-  </si>
-  <si>
-    <t>•	Doctor of Philosopy degree, [Massachusetts Institute of Technology]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/MIT-logo.png}, Cambridge, Massachusettes
+• Used [Linux](https://www.debian.org/), [C programming language](https://www.cprogramming.com/books/ritchie.html), and [Visio](https://www.microsoft.com/en-us/microsoft-365/visio/flowchart-software).</t>
+  </si>
+  <si>
+    <t>Warner Brothers</t>
+  </si>
+  <si>
+    <t>Data Laboratory</t>
+  </si>
+  <si>
+    <t>• As a senior full stack developer for [NuSkin](https://www.nuskin.com/us/en/, an international company known for its excellent  skin and beauty products I created new [Vue.js](https://vuejs.org/), [Nuxt](https://nuxt.com/), and [Vuetify](https://vuetifyjs.com/en/) components using [Bash], [Linux], [GitHub], [NodeJS], [HTML] and [CSS].  
+• Internationalized content using [Adobe Experience Cloud](https://business.adobe.com/).</t>
+  </si>
+  <si>
+    <t>• As a senior data engineer for SeniorLink's [Vela project]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/Vela-150x126.png} a homeservices support platform, helped create [ETL](https://aws.amazon.com/what-is/etl/) processes using [Amazon Kinesis](https://aws.amazon.com/pm/kinesis/), [Python], [PySpark](https://spark.apache.org/), and [Amazon Data Pipeline](https://docs.aws.amazon.com/datapipeline/latest/DeveloperGuide/what-is-datapipeline.html) to load structured event data from [PostgreSQL] databases into [Redshift](https://aws.amazon.com/pm/redshift/). 
+• Saved data to [Amazon S3] using [Amazon Kinesis] and triggered [Amazon Lambda](https://docs.aws.amazon.com/lambda/) jobs to aggregate steaming event data into [schema-on-read] file formats, [Apache Avro](https://avro.apache.org/) and [Apache Parquet](https://parquet.apache.org/).
+• Steered efforts in creating a [Data Lake](https://aws.amazon.com/big-data/datalakes-and-analytics/datalakes/) using [PostgreSQL] and [FlyWay](https://flywaydb.org/) with [Python] and [PySpark](https://spark.apache.org/docs/latest/api/python/index.html) pre-processing on [EC2 instances] using shared [Amazon EFS](https://zesty.co/blog/ebs-vs-efs-which-is-right) for staged storage.
+• Used streaming event messages queued in [RabbitMQ](https://docs.aws.amazon.com/amazon-mq/latest/developer-guide/working-with-rabbitmq.html) and [Amazon Kinesis] to build [type-2 slowly changing dimensions] and accumulative facts tables. 
+• Designed and implemented a custom [star-schema warehouse](https://www.databricks.com/glossary/star-schema) and [ETL] processes to [de-normalize](https://en.wikipedia.org/wiki/Denormalization) and load data into [Redshift](https://aws.amazon.com/redshift/) data warehouse for BI reporting using [Tableau](https://www.tableau.com/).
+• [Test-driven development](https://www.pluralsight.com/blog/software-development/tdd-vs-bdd) using [Bash], [Linux], [Python], [PyCharm], [PyTest], [Unit-test], [GitHub], [Jira], and [Jenkins](https://www.jenkins.io/).</t>
+  </si>
+  <si>
+    <t>• Co-founded [ClipFile]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/clipfile-infrastructure-150x150.png}, a company that envisioned building a web destination where users could easily record and share their favorite pieces of content like facts, authored stories, quotes, articles, chapters, or personal thoughts, as a way of concretely defining their personal [mindset]{https://sourcesofinsight.com/wp-content/uploads/2014/04/Mindset-768x505.jpg}(https://sourcesofinsight.com/what-is-mindset/).
+• Implemented [fuzzy matching](https://nanonets.com/blog/fuzzy-matching-fuzzy-logic/), [word clustering](https://www.ilc.cnr.it/EAGLES96/rep2/node37.html#:~:text=Word%20clustering%20is%20a%20technique,to%20information%20retrieval%20and%20filtering.), [semantic similarity scores](https://towardsdatascience.com/semantic-similarity-using-transformers-8f3cb5bf66d6), and [collaborative filtering](https://www.hindawi.com/journals/aai/2009/421425/) to help users find content that matched or differed from thieir own mindset.
+• Launched a novel [SaaS] using [Amazon Web Services] that let individuals and content creators search and share mindsets.
+• Conceptualized patented technology by designing and implementing a fuil-stack consumer-facing content management system that supported tuned matching among selected attributes.
+• [Java], [J2EE], [JSP], [Servlets], [Spring], [Amazon services], [JavaScript], [JQuery], [HTML], [CSS], [JUnit], [JMeter], [JProfile].
+• Utilized [REST], [Swagger], [Apache Shiro](https://shiro.apache.org/), [Eclipse IDE](https://www.eclipse.org/home/whatis/), [Apache Maven](https://maven.apache.org/what-is-maven.html), [Apache Ant](https://ant.apache.org/), [GitHub], [Hibernate], [Amazon SimpleDB](https://aws.amazon.com/simpledb/), [Linux](https://www.centos.org/), [Apache Tomcat](https://tomcat.apache.org/), [Bash], [Linux], [Jetty](https://projects.eclipse.org/projects/rt.jetty), and [Spring MVC](https://docs.spring.io/spring-framework/reference/web/webmvc.html).
+• Served as co-founder and co-authored [four patents](https://www.freepatentsonline.com/y2013/0325870.html).</t>
+  </si>
+  <si>
+    <t>• As lead software developer, built a CD-ROM-based home design application for selecting premium home design products for previewing in the context of images of any household rooms. 
+• Built the prototype using Adobe Photoshop and [Macromedia Director](https://macromedia.fandom.com/wiki/Macromedia_Director).
+• Built the actual application using using [Bash], [Linux], [Java] and [Marimba Bongo](https://www.thriftbooks.com/w/official-marimba-guide-to-bongo_danny-goodman/2574616/#edition=58026223&amp;idiq=42367912) widget layout tool.
+• Updates for the self-updating application were delivered over the internet using [Marimba Castanet](https://www.infoworld.com/article/2076707/marimba-launches-new-castanet-with-a-less-java-centric-focus.html) push-technology.</t>
+  </si>
+  <si>
+    <t>• Front-end software developer of a reverse kinametics path planning system for multi-axis industrial robots for [Cimmetrix]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/Cimetrix-PDF-combined-logo-150x100.png}.
+• Technologies used include [Bash], [Linux], [C programming language], [Bash](https://en.wikipedia.org/wiki/Bourne_shell), [X11] , [Xt toolkit intrinsics](https://en.wikipedia.org/wiki/X_Toolkit_Intrinsics), [Silicon Graphics Irix](https://en.wikipedia.org/wiki/Silicon_Graphics), and [HP-UX](https://en.wikipedia.org/wiki/HP-UX).</t>
+  </si>
+  <si>
+    <t>•  AMI (https://amientertainment.com/) was the internet-music distribution incarnation of Rowe International.  
+•  As a Sierra Vista Group project manager and technical lead, I helped design and implement their system for making monthly ACH royalty payments to music copyright owners for mechanical and performance licensing rights.
+•  Used [FileMaker Pro](https://www.claris.com/filemaker/), [Bash], [Linux], [HTML], [CSS], [JavaScript], [Java], and [Visio](https://www.microsoft.com/en-us/microsoft-365/visio/flowchart-software).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">•  [Rowe International](https://pitchbook.com/profiles/company/13178-08) was the leading manufacturer of music jukeboxes. 
+•  Sierra Vista Group was consulted to assess their available technologies and create a plan to build their back-end systems to let them become a leading provider of internet-based music.
+•  As project manager and technical lead created the project plan and led the development of a full-stack web application used by  jukebox owners and Rowe sales and marketing.
+•  Used [Java], [Bash], [Linux], [HTML], [CSS], [JavaScript], [ObjectDesign](https://object.design/), [MySQL](https://www.mysql.com/), and [Adobe Photoshop](https://www.adobe.com/products/photoshop.html). 
+</t>
+  </si>
+  <si>
+    <t>•	Doctor of Philosopy degree, [MIT]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/MIT-logo.png}, Cambridge, Massachusettes
 •	Media Laboratory, Media Arts and Sciences
 •	Took courses in machine vision, signals and systems, digital signal processing, and stochastics.
 •	Helped build the operating system for the [Cheops multi-processor system](http://alumni.media.mit.edu/~wad/cheops_CSVT/cheops.html) used for digital video research and for holographic video
@@ -281,99 +324,56 @@
 •	“Semiautomatic Camera Lens Calibration from Partially Known Structure”, Shawn Becker, MIT Media Lab Reports, 1994
 •	[“Formulating a scene probability equation to differentiate the effects of shape &amp; albedo on image brightness.”](https://www.researchgate.net/publication/2668457_Formulating_a_Scene_Probability_Equation_to_Differentiate_the_Effects_of_Shape_and_Albedo_on_Image_Brightness) Shawn Becker, MIT Media Lab Reports, 1994
 •	“Computation of some projective-chirplet-transform &amp; metaplectic-chirplet-transform subspaces, with applications in image processing.” Steve Mann &amp; Shawn Becker, DSP World Symposium, Boston, Massachusetts, November 1992.
-• [C programming language], [TclTk], [X11], [HTML], [JavaScript],[CSS],[XMotif], [bash], [Linux]</t>
-  </si>
-  <si>
-    <t>• As a senior full stack developer for [NuSkin](https://www.nuskin.com/us/en/, an international company known for its excellent  skin and beauty products I created new [Vue.js](https://vuejs.org/), [Nuxt](https://nuxt.com/), and [Vuetify](https://vuetifyjs.com/en/) components using [bash], [Linux], [GitHub], [NodeJS], [HTML] and [CSS].  
-• Internationalized content using [Adobe Experience Cloud](https://business.adobe.com/).</t>
-  </si>
-  <si>
-    <t>• As co-founder and CTO, designed and led the development of a public website used by discerning home designers and builders called [HomePortfolio.com](https://homeportfolio.com/). 
+• [C programming language], [TclTk], [X11], [HTML], [JavaScript],[CSS],[XMotif], [Bash], [Linux]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• [Eleven LLC](https://www.eleven.net/) built mobile apps used by beverage industry distributors to help manage placement  of their products in the shelves and coolers in retail locations. The work done by the Sierra Vista Group was instrumental in their company being acquired by [Trimble](https://help.trimblegeospatial.com/TMM/Home.htm). 
+• As the architect and team lead, we used [Java], [Bash], [GitHub], [Linux], and  [JBoss](https://developers.redhat.com/products/eap/overview) message-oriented middleware platform, [Sybase Anywhere](https://texas.gs.shi.com/Product/30451452/Sybase-SQL-Anywhere-Advanced-Edition) for the client/server based database, and [Windows Mobile](https://en.wikipedia.org/wiki/Windows_Mobile_5.0) running on ruggedized mobile devices. </t>
+  </si>
+  <si>
+    <t>• As co-founder and CTO, designed and led the development of a public website used by discerning home designers and builders called [HomePortfolio](https://HomePortfolio/). 
 • Hired a staff of  10 software and databases developers. 
 • Worked with data acquisition team to scan and tag over 700,000 premium home design products from over 2,000 manufactures and vendors.
 • Designed datamodel and data entry tools for category-specific product attribution. 
 • Helped extended the business model to provide online product selection tools for participating vendors and manufacturers.
 • Instrumental in raising over $70M in venture capital. 
-• Used [Oracle], [ATG Dyanamo]( https://docs.oracle.com/cd/E24152_01/Platform.10-1/ATGPersBusinessGuide/html/s0102dynamoapplicationframework01.html), [Java], [Akamai]{https://www.hiclipart.com/free-transparent-background-png-clipart-zkmsn}(https://www.akamai.com/), [WebTrends](https://www.webtrends.com/), [FileMakerPro], [ImageMagik](https://imagemagick.org/index.php), [bash], [Linux], [HTML], [JavaScript], [CSS], and [Omnigraffle](https://www.omnigroup.com/omnigraffle) for data modeling and workflow designs.</t>
-  </si>
-  <si>
-    <t>• As lead software developer, built a CD-ROM-based home design application for selecting premium home design products for previewing in the context of images of any household rooms. 
-• Built the prototype using Adobe Photoshop and [Macromedia Director](https://macromedia.fandom.com/wiki/Macromedia_Director).
-• Built the actual application using using [bash], [Linux], [Java] and [Marimba Bongo](https://www.thriftbooks.com/w/official-marimba-guide-to-bongo_danny-goodman/2574616/#edition=58026223&amp;idiq=42367912) widget layout tool.
-• Updates for the self-updating application were delivered over the internet using [Marimba Castanet](https://www.infoworld.com/article/2076707/marimba-launches-new-castanet-with-a-less-java-centric-focus.html) push-technology.</t>
-  </si>
-  <si>
-    <t>• Masters of Science degree, [Brigham Young University]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/BYU-entrance-150x150.jpg}, Provo, Utah
+• Used [Oracle], [ATG Dyanamo]( https://docs.oracle.com/cd/E24152_01/Platform.10-1/ATGPersBusinessGuide/html/s0102dynamoapplicationframework01.html), [Java], [Akamai]{https://www.hiclipart.com/free-transparent-background-png-clipart-zkmsn}(https://www.akamai.com/), [WebTrends](https://www.webtrends.com/), [FileMakerPro], [ImageMagik](https://imagemagick.org/index.php), [Bash], [Linux], [HTML], [JavaScript], [CSS], and [Omnigraffle](https://www.omnigroup.com/omnigraffle) for data modeling and workflow designs.</t>
+  </si>
+  <si>
+    <t>• Masters of Science degree, [BYU]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/BYU-entrance-150x150.jpg}, Provo, Utah
 Took all courses required for both bachelors and masters degrees in Computer Science
 • Thesis project [“Interactive Measurement of Three-Dimensional Objects Using a Depth Buffer &amp; Linear Probe.”](https://dl.acm.org/doi/pdf/10.1145/108360.108446) CS MS Thesis, Shawn Becker, William A. Barrett &amp; Dan R. Olsen, ACM Transactions on Graphics, Vol. 10, No. 2, April 1991
-• Top Research Presentation – New Tech Research Conference - Brigham Young University – Provo, UT – March 1990
+• Top Research Presentation – New Tech Research Conference - BYU – Provo, UT – March 1990
 • [“Fast Automated Object Detection Using Signature Parsing.”](https://www.spiedigitallibrary.org/conference-proceedings-of-spie/1192/1/Fast-Automated-Object-Detection-Using-Signature-Parsing/10.1117/12.969720.short) Tim Heaton; Shawn Becker; Kelley Anderson; William Barrett: Proceedings Volume 1192, Intelligent Robots &amp; Computer Vision VIII: Algorithms &amp; Techniques; (1990) https://doi.org/10.1117/12.969720
 • [“Probabilistic Segmentation of Myocardial Tissue by Deterministic Relaxation.”](https://scholarsarchive.byu.edu/cgi/viewcontent.cgi?article=1737&amp;context=facpub) Jerome A. Broekhuijsen, Shawn C. Becker, &amp; William A. Barrett: IEEE Proceedings of Computers in Cardiology, pp. 99-12, Jerusalem, September 1989.
 • [“Interactive Measurement of three-Dimensional Cardiac Morphology.”]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/BYU-MS-CS-Skull-Cross-Section-1.jpeg}(https://scholarsarchive.byu.edu/cgi/viewcontent.cgi?article=1736&amp;context=facpub) Shawn C Becker, William A Barrett, October 1989, DOI: 10.1109/CIC.1989.130586, Conference: Computers in Cardiology.
-• [C programming language], [bash], [Linux], [XMotif], and [X11].</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• [Eleven LLC](https://www.eleven.net/) built mobile apps used by beverage industry distributors to help manage placement  of their products in the shelves and coolers in retail locations. The work done by the Sierra Vista Group was instrumental in their company being acquired by [Trimble Mobile Solutions](https://help.trimblegeospatial.com/TMM/Home.htm). 
-• As the architect and team lead, we used [Java], [bash], [GitHub], [Linix], and  [JBoss](https://developers.redhat.com/products/eap/overview) message-oriented middleware platform, [Sybase Anywhere](https://texas.gs.shi.com/Product/30451452/Sybase-SQL-Anywhere-Advanced-Edition) for the client/server based database, and [Windows Mobile](https://en.wikipedia.org/wiki/Windows_Mobile_5.0) running on ruggedized mobile devices. </t>
-  </si>
-  <si>
-    <t>•  AMI (https://amientertainment.com/) was the internet-music distribution incarnation of Rowe International.  
-•  As a Sierra Vista Group project manager and technical lead, I helped design and implement their system for making monthly ACH royalty payments to music copyright owners for mechanical and performance licensing rights.
-•  Used [FileMaker Pro](https://www.claris.com/filemaker/), [bash], [Linux], [HTML], [CSS], [JavaScript], [Java], and [Visio](https://www.microsoft.com/en-us/microsoft-365/visio/flowchart-software).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">•  [Rowe International](https://pitchbook.com/profiles/company/13178-08) was the leading manufacturer of music jukeboxes. 
-•  Sierra Vista Group was consulted to assess their available technologies and create a plan to build their back-end systems to let them become a leading provider of internet-based music.
-•  As project manager and technical lead created the project plan and led the development of a full-stack web application used by  jukebox owners and Rowe sales and marketing.
-•  Used [Java], [bash], [Linux], [HTML], [CSS], [JavaScript], [ObjectDesign](https://object.design/), [MySQL](https://www.mysql.com/), and [Adobe Photoshop](https://www.adobe.com/products/photoshop.html). 
-</t>
+• [C programming language], [Bash], [Linux], [XMotif], and [X11].</t>
   </si>
   <si>
     <t>• As a senior software engineer at [BigR.io]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/Bigr.io_-150x106.png} I used [Amazon microservices] for custom voice-based [natural language processing] applications.
-• Used [Apache ActiveMQ](https://activemq.apache.org/), [Swagger](https://swagger.io/), [JSON], [Jackson](url), [AOP](https://www.baeldung.com/spring-aop), [Eclipse], [Maven], [GitHub], [Jira], and [Jenkins].
-• [Java], [J2EE], [Servlets], [Spring], [SpringBoot], [JAX-RS], [bash], [Linux], [JUnit], [JMeter], and [JProfile]</t>
-  </si>
-  <si>
-    <t>• As a senior data engineer in the data cyber security team of the [Cigna Group](https://www.thecignagroup.com/) created a [REST API](url) using [Postman](https://www.postman.com/), [bash], [Linux], and [OpenAPI](https://openapi-generator.tech/) for pulling credentials from the [CyberArk identity security platform](https://www.cyberark.com/) using [mutual TLS SSL authentication](https://docs.solace.com/Security/Two-Way-SSL-Authentication.htm) with [Amazon API Gateway](https://docs.aws.amazon.com/apigateway/). 
-•  Migrated a suite of legacy data pipeline [Python] elements running on the [Unity IoC platform](http://unitycontainer.org/articles/introduction.html) to pull credentials from the CyberArk service at runtime rather than using [Fernet](https://cryptography.io/en/latest/fernet/) encrypted local files. 
+• Used [Apache ActiveMQ](https://activemq.apache.org/), [Swagger](https://swagger.io/), [JSON], [Jackson](url), [AOP](https://www.baeldung.com/spring-aop), [Eclipse], [Maven], [GitHub], [Jira], [PostgreSQL], and [Jenkins].
+• [Java], [J2EE], [Servlets], [Spring], [SpringBoot], [JAX-RS], [Bash], [Linux], [JUnit], [JMeter], and [JProfile]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As a senior software engineer for Data Laboratory, an internet company that provides daily lead reports for independent real-estage agents world-wide, I  [containerized] legacy web applications using [Bash], [Linux], [GitHub], [Docker](https://www.docker.com/) and [Amazon Secrets Manager](https://aws.amazon.com/secrets-manager/). 
+• Updated legacy web apps using [Bash], [Linux], [HTML], [CSS], [JavaScript], [PostgreSQL], [NGINX], and [OpenSSL].
+• Documented existing data architecture as [ERDs](https://www.lucidchart.com/pages/er-diagrams) using [DBeaver Enterprise](https://dbeaver.com/dbeaver-enterprise/). </t>
+  </si>
+  <si>
+    <t>• As a senior data engineer for [Angel Studios](https://www.angel.com/home), a streaming media service that offers family-friendly entertainment that amplifies light, with titles including The Chosen, Dry Bar Comedy, and Tuttle Twins.
+• Used [Python], [GitHub], [Pandas], [Numpy], [Keras], [Bash], [Linux], [PostgreSQL], and [Jupyter](https://jupyter.org/) to build and tune hyperparameters of a [convolutional neural network](https://towardsdatascience.com/a-comprehensive-guide-to-convolutional-neural-networks-the-eli5-way-3bd2b1164a53) with [supervised learning] on [Amazon Sagemaker](https://aws.amazon.com/pm/sagemaker/) to classify movie frames from episodic programs stored in [Amazon S3](https://aws.amazon.com/s3/storage-classes). 
+• Built web client apps using [Python] with [Postman](https://www.postman.com/) that made [REST] requests to pull monthly usage data from various web marketing partners like [FaceBook Marketing](https://www.quora.com/What-is-Facebook-Marketing-1), [Google Play](https://play.google/howplayworks/) , and [Vimeo](https://vimeo.com/). 
+• Worked with [Segment customer data platform](https://segment.com/customer-data-platform/), [Excel], and [Tableau] to create scheduled reports for the company's sales and finance teams.</t>
+  </si>
+  <si>
+    <t>• As a senior data engineer in the analytics team of [Warner Brothers](https://warnerbrosgames.com/) Division, I implemented high-volume pipeline integrations shuffling game telemetry and [user PII data] between WB-distributed consumer games and [marketing service platforms] via [Segment customer data platform](https://segment.com/customer-data-platform/) using [Kafka](https://aws.amazon.com/msk/), [Redshift](https://aws.amazon.com/redshift/), and [Apache Airflow](https://airflow.apache.org). 
+• Employed [Python], [GitHub], [Bash], [Linux], [Amazon Glue](https://aws.amazon.com/glue/) and [Apache Airflow](https://airflow.apache.org/) for external 3rd-party integrations and internal dev-ops integrations with [Jenkins], [PostgreSQL], [DataDog](https://www.datadoghq.com/), and [ZenDesk](https://zendesk.com) 
+• Integrated with [Google BigQuery data warehouse](https://cloud.google.com/bigquery using  [Apache Airflow](https://aws.amazon.com/managed-workflows-for-apache-airflow/), [Amazon S3], and [Redshift](https://aws.amazon.com/redshift/).</t>
+  </si>
+  <si>
+    <t>• As a senior data engineer in the data cyber security team of the [Cigna Group](https://www.thecignagroup.com/) created a [REST](url) using [Postman](https://www.postman.com/), [Bash], [Linux], and [OpenAPI](https://openapi-generator.tech/) for pulling credentials from the [CyberArk identity security platform](https://www.cyberark.com/) using [mutual TLS SSL authentication](https://docs.solace.com/Security/Two-Way-SSL-Authentication.htm) with [API Gateway](https://docs.aws.amazon.com/apigateway/). 
+•  Migrated a suite of legacy data pipeline [Python] elements running on the [Unity IoC platform](http://unitycontainer.org/articles/introduction.html) with [PostgreSQL] to pull credentials from the CyberArk service at runtime rather than using [Fernet](https://cryptography.io/en/latest/fernet/) encrypted local files. 
 •  Upgraded [GitHub] apps to use [Jenkins](https://docs.aws.amazon.com/apigateway/) CI/CD pipeline for build, applying sofware and cyber-secutity code checks, and on-prem server installation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• As a senior software engineer for Greenseed Tech, an internet company that provides daily lead reports for independent real-estage agents world-wide, I  [containerized] legacy web applications using [bash], [Linux], [GitHub], [Docker](https://www.docker.com/) and [Amazon Secrets Manager](https://aws.amazon.com/secrets-manager/). 
-• Updated legacy web apps using [bash], [Linux], [HTML], [CSS], [JavaScript], [NGINX], and [OpenSSL].
-• Documented existing data architecture as [ERDs](https://www.lucidchart.com/pages/er-diagrams) using [DBeaver Enterprise](https://dbeaver.com/dbeaver-enterprise/). </t>
-  </si>
-  <si>
-    <t>• Co-founded [ClipFile]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/clipfile-infrastructure-150x150.png}, a company that envisioned building a web destination where users could easily record and share their favorite pieces of content like facts, authored stories, quotes, articles, chapters, or personal thoughts, as a way of concretely defining their personal [mindset]{https://sourcesofinsight.com/wp-content/uploads/2014/04/Mindset-768x505.jpg}(https://sourcesofinsight.com/what-is-mindset/).
-• Implemented [fuzzy matching](https://nanonets.com/blog/fuzzy-matching-fuzzy-logic/), [word clustering](https://www.ilc.cnr.it/EAGLES96/rep2/node37.html#:~:text=Word%20clustering%20is%20a%20technique,to%20information%20retrieval%20and%20filtering.), [semantic similarity scores](https://towardsdatascience.com/semantic-similarity-using-transformers-8f3cb5bf66d6), and [collaborative filtering](https://www.hindawi.com/journals/aai/2009/421425/) to help users find content that matched or differed from thieir own mindset.
-• Launched a novel [SaaS] using [Amazon Web Services] that let individuals and content creators search and share mindsets.
-• Conceptualized patented technology by designing and implementing a fuil-stack consumer-facing content management system that supported tuned matching among selected attributes.
-• [Java], [J2EE], [JSP], [Servlets], [Spring], [Amazon services], [JavaScript], [JQuery], [HTML], [CSS], [JUnit], [JMeter], [JProfile].
-• Utilized [REST API], [Swagger], [Apache Shiro](https://shiro.apache.org/), [Eclipse IDE](https://www.eclipse.org/home/whatis/), [Apache Maven](https://maven.apache.org/what-is-maven.html), [Apache Ant](https://ant.apache.org/), [GitHub], [Hibernate], [Amazon SimpleDB](https://aws.amazon.com/simpledb/), [CentOS Linux](https://www.centos.org/), [Apache Tomcat](https://tomcat.apache.org/), [bash], [Linux], [Jetty](https://projects.eclipse.org/projects/rt.jetty), and [Spring MVC](https://docs.spring.io/spring-framework/reference/web/webmvc.html).
-• Served as co-founder and co-authored [four patents](https://www.freepatentsonline.com/y2013/0325870.html).</t>
-  </si>
-  <si>
-    <t>• As a senior data engineer in the analytics team of [Warner Brothers Interactive Entertainment](https://warnerbrosgames.com/) Division, I implemented high-volume pipeline integrations shuffling game telemetry and [user PII data] between WB-distributed consumer games and [marketing service platforms] via [Segment customer data platform](https://segment.com/customer-data-platform/) using [Kafka](https://aws.amazon.com/msk/), [Amazon Redshift](https://aws.amazon.com/redshift/), and [Apache Airflow](https://airflow.apache.org). 
-• Employed [Python], [GitHub], [bash], [Linux], [Amazon Glue](https://aws.amazon.com/glue/) and [Apache Airflow](https://airflow.apache.org/) for external 3rd-party integrations and internal dev-ops integrations with [Jenkins], [DataDog](https://www.datadoghq.com/), and [ZenDesk](https://zendesk.com) 
-• Integrated with [Google BigQuery data warehouse](https://cloud.google.com/bigquery using  [Apache Airflow](https://aws.amazon.com/managed-workflows-for-apache-airflow/), [Amazon S3], and [Amazon Redshift](https://aws.amazon.com/redshift/).</t>
-  </si>
-  <si>
-    <t>• Front-end software developer of a reverse kinametics path planning system for multi-axis industrial robots for [Cimmetrix]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/Cimetrix-PDF-combined-logo-150x100.png}.
-• Technologies used include [bash], [Linux], [C programming language], [bash](https://en.wikipedia.org/wiki/Bourne_shell), [X11] , [Xt toolkit intrinsics](https://en.wikipedia.org/wiki/X_Toolkit_Intrinsics), [Silicon Graphics Irix](https://en.wikipedia.org/wiki/Silicon_Graphics), and [HP-UX](https://en.wikipedia.org/wiki/HP-UX).</t>
-  </si>
-  <si>
-    <t>• As a senior data engineer for [Angel Studios](https://www.angel.com/home), a streaming media service that offers family-friendly entertainment that amplifies light, with titles including The Chosen, Dry Bar Comedy, and Tuttle Twins.
-• Used [Python], [GitHub], [Pandas], [Numpy], [Keras], [bash], [Linux], and [Jupyter](https://jupyter.org/) to build and tune hyperparameters of a [convolutional neural network](https://towardsdatascience.com/a-comprehensive-guide-to-convolutional-neural-networks-the-eli5-way-3bd2b1164a53) with [supervised learning] on [Amazon Sagemaker](https://aws.amazon.com/pm/sagemaker/) to classify movie frames from episodic programs stored in [Amazon S3](https://aws.amazon.com/s3/storage-classes). 
-• Built web client apps using [Python] with [Postman](https://www.postman.com/) that made [REST API] requests to pull monthly usage data from various web marketing partners like [FaceBook Marketing](https://www.quora.com/What-is-Facebook-Marketing-1), [Google Play](https://play.google/howplayworks/) , and [Vimeo](https://vimeo.com/). 
-• Worked with [Segment customer data platform](https://segment.com/customer-data-platform/), [Excel], and [Tableau] to create scheduled reports for the company's sales and finance teams.</t>
-  </si>
-  <si>
-    <t>• As a senior data engineer for SeniorLink's [Vela project]{https://shawn.beckerstudio.com/wp-content/uploads/2023/05/Vela-150x126.png} a homeservices support platform, helped create [ETL](https://aws.amazon.com/what-is/etl/) processes using [Amazon Kinesis](https://aws.amazon.com/pm/kinesis/), [Python], [PySpark](https://spark.apache.org/), and [Amazon Data Pipeline](https://docs.aws.amazon.com/datapipeline/latest/DeveloperGuide/what-is-datapipeline.html) to load structured event data from [PostgreSQL] databases into [Amazon Redshift](https://aws.amazon.com/pm/redshift/). 
-• Saved data to [Amazon S3] using [Amazon Kinesis] and triggered [Amazon Lambda](https://docs.aws.amazon.com/lambda/) jobs to aggregate steaming event data into [schema-on-read] file formats, [Apache Avro](https://avro.apache.org/) and [Apache Parquet](https://parquet.apache.org/).
-• Steered efforts in creating a [Data Lake](https://aws.amazon.com/big-data/datalakes-and-analytics/datalakes/) using [PostgreSQL] and [FlyWay](https://flywaydb.org/) with [Python] and [PySpark](https://spark.apache.org/docs/latest/api/python/index.html) pre-processing on [EC2 instances] using shared [Amazon EFS](https://zesty.co/blog/ebs-vs-efs-which-is-right) for staged storage.
-• Used streaming event messages queued in [RabbitMQ](https://docs.aws.amazon.com/amazon-mq/latest/developer-guide/working-with-rabbitmq.html) and [Amazon Kinesis] to build [type-2 slowly changing dimensions] and accumulative facts tables. 
-• Designed and implemented a custom [star-schema warehouse](https://www.databricks.com/glossary/star-schema) and [ETL] processes to [de-normalize](https://en.wikipedia.org/wiki/Denormalization) and load data into [Amazon Redshift](https://aws.amazon.com/redshift/) data warehouse for BI reporting using [Tableau](https://www.tableau.com/).
-• [Test-driven development](https://www.pluralsight.com/blog/software-development/tdd-vs-bdd) using [bash], [Linux], [Python], [PyCharm], [PyTest], [Unit-test], [GitHub], [Jira], and [Jenkins](https://www.jenkins.io/).</t>
   </si>
 </sst>
 </file>
@@ -963,7 +963,7 @@
     </row>
     <row r="2" spans="1:10" ht="160" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>10</v>
@@ -972,7 +972,7 @@
         <v>45047</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E2" s="8">
         <v>3</v>
@@ -985,18 +985,18 @@
       </c>
       <c r="H2" s="9"/>
       <c r="I2" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="176" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="C3" s="7">
         <v>44805</v>
@@ -1008,25 +1008,25 @@
         <v>2</v>
       </c>
       <c r="F3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="H3" s="11"/>
       <c r="I3" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="192" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="7">
         <v>44501</v>
@@ -1038,25 +1038,25 @@
         <v>1</v>
       </c>
       <c r="F4" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="96" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="C5" s="7">
         <v>44136</v>
@@ -1068,25 +1068,25 @@
         <v>2</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6" s="7">
         <v>43770</v>
@@ -1098,25 +1098,25 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H6" s="14"/>
       <c r="I6" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="320" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7" s="7">
         <v>42795</v>
@@ -1128,25 +1128,25 @@
         <v>2</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H7" s="15"/>
       <c r="I7" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C8" s="7">
         <v>42705</v>
@@ -1158,25 +1158,25 @@
         <v>1</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H8" s="16"/>
       <c r="I8" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="350" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C9" s="7">
         <v>40575</v>
@@ -1188,25 +1188,25 @@
         <v>2</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H9" s="17"/>
       <c r="I9" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="192" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C10" s="7">
         <v>37561</v>
@@ -1218,25 +1218,25 @@
         <v>1</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H10" s="18"/>
       <c r="I10" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="224" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C11" s="7">
         <v>35827</v>
@@ -1248,25 +1248,25 @@
         <v>1</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H11" s="19"/>
       <c r="I11" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="144" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12" s="7">
         <v>35217</v>
@@ -1281,11 +1281,11 @@
         <v>11</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H12" s="9"/>
       <c r="I12" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J12" s="10" t="s">
         <v>82</v>
@@ -1293,10 +1293,10 @@
     </row>
     <row r="13" spans="1:10" ht="335" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C13" s="7">
         <v>33117</v>
@@ -1308,25 +1308,25 @@
         <v>2</v>
       </c>
       <c r="F13" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="304" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C14" s="7">
         <v>32021</v>
@@ -1338,25 +1338,25 @@
         <v>2</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="H14" s="12"/>
       <c r="I14" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C15" s="7">
         <v>32295</v>
@@ -1368,25 +1368,25 @@
         <v>3</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H15" s="13"/>
       <c r="I15" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="112" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C16" s="7">
         <v>39417</v>
@@ -1398,25 +1398,25 @@
         <v>2</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H16" s="20"/>
       <c r="I16" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J16" s="21" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="128" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="112" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C17" s="7">
         <v>38749</v>
@@ -1428,25 +1428,25 @@
         <v>2</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H17" s="22"/>
       <c r="I17" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J17" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="112" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C18" s="7">
         <v>38384</v>
@@ -1458,25 +1458,25 @@
         <v>2</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H18" s="23"/>
       <c r="I18" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C19" s="7">
         <v>38018</v>
@@ -1488,25 +1488,25 @@
         <v>2</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H19" s="24"/>
       <c r="I19" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="144" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C20" s="7">
         <v>37681</v>
@@ -1518,17 +1518,17 @@
         <v>2</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H20" s="25"/>
       <c r="I20" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J20" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
use first day of next month when job[end_year]='CURRENT_DATE'
</commit_message>
<xml_diff>
--- a/static_content/jobs/jobs.xlsx
+++ b/static_content/jobs/jobs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sbecker11/workspace-parallax/flock-of-postcards/static_content/jobs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA857FE2-748A-BB42-A888-8FDC84289780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D6A0FD-33A2-2143-ACCB-51085389D7CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-56200" yWindow="280" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60000" yWindow="-14480" windowWidth="33600" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="jobs" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="99">
   <si>
     <t>role</t>
   </si>
@@ -357,20 +357,36 @@
 • Documented existing data architecture as [ERDs](https://www.lucidchart.com/pages/er-diagrams) using [DBeaver Enterprise](https://dbeaver.com/dbeaver-enterprise/). </t>
   </si>
   <si>
-    <t>• As a senior data engineer for [Angel Studios](https://www.angel.com/home), a streaming media service that offers family-friendly entertainment that amplifies light, with titles including The Chosen, Dry Bar Comedy, and Tuttle Twins.
+    <t>Fannie Mae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senior Data / Machine Learning Engineer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Introductory phase in new role as senior data / machine learning engineer in the Risk &amp; Corporate Systems team at Fannie Mae GSE 
+</t>
+  </si>
+  <si>
+    <t>#006900</t>
+  </si>
+  <si>
+    <t>• Senior data engineer for [Angel Studios](https://www.angel.com/home), a streaming media service that offers family-friendly entertainment that amplifies light, with titles including The Chosen, Dry Bar Comedy, and Tuttle Twins.
 • Used [Python], [GitHub], [Pandas], [Numpy], [Keras], [Bash], [Linux], [PostgreSQL], and [Jupyter](https://jupyter.org/) to build and tune hyperparameters of a [convolutional neural network](https://towardsdatascience.com/a-comprehensive-guide-to-convolutional-neural-networks-the-eli5-way-3bd2b1164a53) with [supervised learning] on [Amazon Sagemaker](https://aws.amazon.com/pm/sagemaker/) to classify movie frames from episodic programs stored in [Amazon S3](https://aws.amazon.com/s3/storage-classes). 
 • Built web client apps using [Python] with [Postman](https://www.postman.com/) that made [REST] requests to pull monthly usage data from various web marketing partners like [FaceBook Marketing](https://www.quora.com/What-is-Facebook-Marketing-1), [Google Play](https://play.google/howplayworks/) , and [Vimeo](https://vimeo.com/). 
 • Worked with [Segment customer data platform](https://segment.com/customer-data-platform/), [Excel], and [Tableau] to create scheduled reports for the company's sales and finance teams.</t>
   </si>
   <si>
-    <t>• As a senior data engineer in the analytics team of [Warner Brothers](https://warnerbrosgames.com/) Division, I implemented high-volume pipeline integrations shuffling game telemetry and [user PII data] between WB-distributed consumer games and [marketing service platforms] via [Segment customer data platform](https://segment.com/customer-data-platform/) using [Kafka](https://aws.amazon.com/msk/), [Redshift](https://aws.amazon.com/redshift/), and [Apache Airflow](https://airflow.apache.org). 
-• Employed [Python], [GitHub], [Bash], [Linux], [Amazon Glue](https://aws.amazon.com/glue/) and [Apache Airflow](https://airflow.apache.org/) for external 3rd-party integrations and internal dev-ops integrations with [Jenkins], [PostgreSQL], [DataDog](https://www.datadoghq.com/), and [ZenDesk](https://zendesk.com) 
-• Integrated with [Google BigQuery data warehouse](https://cloud.google.com/bigquery using  [Apache Airflow](https://aws.amazon.com/managed-workflows-for-apache-airflow/), [Amazon S3], and [Redshift](https://aws.amazon.com/redshift/).</t>
-  </si>
-  <si>
-    <t>• As a senior data engineer in the data cyber security team of the [Cigna Group](https://www.thecignagroup.com/) created a [REST](url) using [Postman](https://www.postman.com/), [Bash], [Linux], and [OpenAPI](https://openapi-generator.tech/) for pulling credentials from the [CyberArk identity security platform](https://www.cyberark.com/) using [mutual TLS SSL authentication](https://docs.solace.com/Security/Two-Way-SSL-Authentication.htm) with [API Gateway](https://docs.aws.amazon.com/apigateway/). 
-•  Migrated a suite of legacy data pipeline [Python] elements running on the [Unity IoC platform](http://unitycontainer.org/articles/introduction.html) with [PostgreSQL] to pull credentials from the CyberArk service at runtime rather than using [Fernet](https://cryptography.io/en/latest/fernet/) encrypted local files. 
-•  Upgraded [GitHub] apps to use [Jenkins](https://docs.aws.amazon.com/apigateway/) CI/CD pipeline for build, applying sofware and cyber-secutity code checks, and on-prem server installation.</t>
+    <t>• As a senior data engineer in the data cyber security team of the [Cigna Group](https://www.thecignagroup.com/) created a [REST API] using [Postman], [Bash], [Linux], and [OpenAPI] for pulling credentials from [CyberArk](https://www.cyberark.com/) using [OpenSSL] with [mutual TLS SSL authentication](https://docs.solace.com/Security/Two-Way-SSL-Authentication.htm) via [API Gateway]. 
+•  Migrated a suite of legacy [ETL][data pipeline] [Python] elements running on the [Unity IoC platform] with [PostgreSQL] and [S3] to pull credentials from the [CyberArk] identity service at runtime rather than using [Fernet](https://cryptography.io/en/latest/fernet/) encrypted local files. 
+•  Upgraded [GitHub] apps to use [Jenkins](https://docs.aws.amazon.com/apigateway/) [CI/CD pipeline] for build, applying software and cyber-security code checks, and on-prem server installation.</t>
+  </si>
+  <si>
+    <t>• As a senior data engineer in the analytics team of [Warner Brothers](https://warnerbrosgames.com/) Division, implemented high-volume [ETL] [data pipeline] [integrations] transforming and sharing  game telemetry and [user PII data] between WB-distributed consumer games and [marketing service platforms] via [Segment customer data platform](https://segment.com/customer-data-platform/) using [Kafka](https://aws.amazon.com/msk/), [Amazon S3], [Redshift](https://aws.amazon.com/redshift/), and [Apache Airflow](https://airflow.apache.org). 
+• Employed [Python], [GitHub], [Bash], [Linux], [Amazon Glue](https://aws.amazon.com/glue/) and [Apache Airflow](https://airflow.apache.org/) for external [3rd-party integrations] and internal dev-ops integrations with [Jenkins], [PostgreSQL], [DataDog](https://www.datadoghq.com/),  [ZenDesk](https://zendesk.com). and [Tableau].
+• Integrated with [Google BigQuery](https://cloud.google.com/bigquery using  [Apache Airflow](https://aws.amazon.com/managed-workflows-for-apache-airflow/), [Amazon S3], and [Redshift](https://aws.amazon.com/redshift/).</t>
+  </si>
+  <si>
+    <t>CURRENT_DATE</t>
   </si>
 </sst>
 </file>
@@ -402,7 +418,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -482,6 +498,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF228B22"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF006900"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -519,7 +541,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -607,6 +629,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,6 +639,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF006900"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -913,7 +943,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.1640625" style="26" bestFit="1" customWidth="1"/>
@@ -958,29 +988,29 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="160" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="C2" s="7">
-        <v>45047</v>
-      </c>
-      <c r="D2" s="7">
-        <v>45277</v>
+        <v>45339</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="E2" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>11</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" s="9"/>
+        <v>94</v>
+      </c>
+      <c r="H2" s="30"/>
       <c r="I2" s="6" t="s">
         <v>63</v>
       </c>
@@ -988,543 +1018,573 @@
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="176" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="144" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>76</v>
+        <v>10</v>
       </c>
       <c r="C3" s="7">
-        <v>44805</v>
+        <v>45047</v>
       </c>
       <c r="D3" s="7">
-        <v>45047</v>
+        <v>45277</v>
       </c>
       <c r="E3" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="11"/>
+        <v>12</v>
+      </c>
+      <c r="H3" s="9"/>
       <c r="I3" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="192" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="176" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="C4" s="7">
-        <v>44501</v>
+        <v>44805</v>
       </c>
       <c r="D4" s="7">
-        <v>44805</v>
+        <v>45047</v>
       </c>
       <c r="E4" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="12"/>
+        <v>14</v>
+      </c>
+      <c r="H4" s="11"/>
       <c r="I4" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="96" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="192" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="C5" s="7">
-        <v>44136</v>
+        <v>44501</v>
       </c>
       <c r="D5" s="7">
-        <v>44501</v>
+        <v>44805</v>
       </c>
       <c r="E5" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="13"/>
+        <v>17</v>
+      </c>
+      <c r="H5" s="12"/>
       <c r="I5" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="64" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="96" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="C6" s="7">
-        <v>43770</v>
+        <v>44136</v>
       </c>
       <c r="D6" s="7">
-        <v>44136</v>
+        <v>44501</v>
       </c>
       <c r="E6" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H6" s="14"/>
+        <v>19</v>
+      </c>
+      <c r="H6" s="13"/>
       <c r="I6" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="320" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="C7" s="7">
-        <v>42795</v>
+        <v>43770</v>
       </c>
       <c r="D7" s="7">
-        <v>43770</v>
+        <v>44136</v>
       </c>
       <c r="E7" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H7" s="15"/>
+        <v>22</v>
+      </c>
+      <c r="H7" s="14"/>
       <c r="I7" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="335" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="C8" s="7">
-        <v>42705</v>
+        <v>42795</v>
       </c>
       <c r="D8" s="7">
-        <v>42795</v>
+        <v>43770</v>
       </c>
       <c r="E8" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H8" s="16"/>
+        <v>25</v>
+      </c>
+      <c r="H8" s="15"/>
       <c r="I8" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J8" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="7">
+        <v>42705</v>
+      </c>
+      <c r="D9" s="7">
+        <v>42795</v>
+      </c>
+      <c r="E9" s="8">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="16"/>
+      <c r="I9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="J9" s="10" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="335" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
+    <row r="10" spans="1:10" ht="335" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C10" s="7">
         <v>40575</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D10" s="7">
         <v>42705</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E10" s="8">
         <v>2</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="192" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="7">
-        <v>37561</v>
-      </c>
-      <c r="D10" s="7">
-        <v>40575</v>
-      </c>
-      <c r="E10" s="8">
-        <v>1</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="18"/>
+      <c r="H10" s="17"/>
       <c r="I10" s="6" t="s">
         <v>64</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="224" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="192" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C11" s="7">
-        <v>35827</v>
+        <v>37561</v>
       </c>
       <c r="D11" s="7">
-        <v>37561</v>
+        <v>40575</v>
       </c>
       <c r="E11" s="8">
         <v>1</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="H11" s="19"/>
+        <v>34</v>
+      </c>
+      <c r="H11" s="18"/>
       <c r="I11" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="144" x14ac:dyDescent="0.2">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="224" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C12" s="7">
-        <v>35217</v>
+        <v>35827</v>
       </c>
       <c r="D12" s="7">
-        <v>35827</v>
+        <v>37561</v>
       </c>
       <c r="E12" s="8">
         <v>1</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H12" s="9"/>
+        <v>37</v>
+      </c>
+      <c r="H12" s="19"/>
       <c r="I12" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="335" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="144" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C13" s="7">
-        <v>33117</v>
+        <v>35217</v>
       </c>
       <c r="D13" s="7">
-        <v>35521</v>
+        <v>35827</v>
       </c>
       <c r="E13" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="11"/>
+        <v>40</v>
+      </c>
+      <c r="H13" s="9"/>
       <c r="I13" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="304" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="335" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C14" s="7">
-        <v>32021</v>
+        <v>33117</v>
       </c>
       <c r="D14" s="7">
-        <v>33117</v>
+        <v>35521</v>
       </c>
       <c r="E14" s="8">
         <v>2</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="H14" s="12"/>
+        <v>14</v>
+      </c>
+      <c r="H14" s="11"/>
       <c r="I14" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="304" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
-        <v>72</v>
+        <v>43</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C15" s="7">
-        <v>32295</v>
+        <v>32021</v>
       </c>
       <c r="D15" s="7">
-        <v>32752</v>
+        <v>33117</v>
       </c>
       <c r="E15" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H15" s="13"/>
+        <v>45</v>
+      </c>
+      <c r="H15" s="12"/>
       <c r="I15" s="6" t="s">
         <v>63</v>
       </c>
       <c r="J15" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="7">
+        <v>32295</v>
+      </c>
+      <c r="D16" s="7">
+        <v>32752</v>
+      </c>
+      <c r="E16" s="8">
+        <v>3</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="13"/>
+      <c r="I16" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="J16" s="10" t="s">
         <v>82</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="112" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="7">
-        <v>39417</v>
-      </c>
-      <c r="D16" s="7">
-        <v>40391</v>
-      </c>
-      <c r="E16" s="8">
-        <v>2</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="J16" s="21" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="112" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C17" s="7">
-        <v>38749</v>
+        <v>39417</v>
       </c>
       <c r="D17" s="7">
-        <v>39417</v>
+        <v>40391</v>
       </c>
       <c r="E17" s="8">
         <v>2</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H17" s="22"/>
+        <v>50</v>
+      </c>
+      <c r="H17" s="20"/>
       <c r="I17" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="J17" s="10" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="96" x14ac:dyDescent="0.2">
+      <c r="J17" s="21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="128" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C18" s="7">
-        <v>38384</v>
+        <v>38749</v>
       </c>
       <c r="D18" s="7">
-        <v>38749</v>
+        <v>39417</v>
       </c>
       <c r="E18" s="8">
         <v>2</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="H18" s="23"/>
+        <v>53</v>
+      </c>
+      <c r="H18" s="22"/>
       <c r="I18" s="6" t="s">
         <v>64</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="80" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="96" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C19" s="7">
-        <v>38018</v>
+        <v>38384</v>
       </c>
       <c r="D19" s="7">
-        <v>38384</v>
+        <v>38749</v>
       </c>
       <c r="E19" s="8">
         <v>2</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H19" s="24"/>
+        <v>56</v>
+      </c>
+      <c r="H19" s="23"/>
       <c r="I19" s="6" t="s">
         <v>64</v>
       </c>
       <c r="J19" s="10" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="144" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C20" s="7">
-        <v>37681</v>
+        <v>38018</v>
       </c>
       <c r="D20" s="7">
-        <v>38018</v>
+        <v>38384</v>
       </c>
       <c r="E20" s="8">
         <v>2</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="H20" s="25"/>
+        <v>59</v>
+      </c>
+      <c r="H20" s="24"/>
       <c r="I20" s="6" t="s">
         <v>64</v>
       </c>
       <c r="J20" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="144" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="7">
+        <v>37681</v>
+      </c>
+      <c r="D21" s="7">
+        <v>38018</v>
+      </c>
+      <c r="E21" s="8">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="H21" s="25"/>
+      <c r="I21" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J21" s="10" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>